<commit_message>
Reconstruct D5 publication figures
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/publication/FigD5_6_validation_coverage_source_data.xlsx
+++ b/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/publication/FigD5_6_validation_coverage_source_data.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="outer_refit" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="localization" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monthly_coverage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="risk_coverage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="topological_hops" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monthly_coverage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="risk_coverage" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2720,365 +2721,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>month</t>
+          <t>hop_class</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>sensor_hours</t>
+          <t>n_trials</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>raw_score_coverage</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>report_score_coverage</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>ood_rate</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>L1_rate</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>L2_rate</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>L3_rate</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>D5_raw_median</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>D5_raw_p05</t>
+          <t>fraction</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>0 (correct node)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10416</v>
+        <v>112</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9731182795698925</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.9005376344086021</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.7857142857142857</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.2142857142857143</v>
-      </c>
-      <c r="I2" t="n">
-        <v>3.803353078474338</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1.97904518140716</v>
+        <v>0.6222222222222222</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>1 hop</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10080</v>
+        <v>65</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9722222222222222</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.8347222222222223</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.8172619047619047</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.1827380952380952</v>
-      </c>
-      <c r="I3" t="n">
-        <v>3.372117688407658</v>
-      </c>
-      <c r="J3" t="n">
-        <v>1.617424389235149</v>
+        <v>0.3611111111111111</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2+ hops</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10416</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.9326036866359447</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.0673963133640553</v>
-      </c>
-      <c r="I4" t="n">
-        <v>3.068031596388653</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1.458730046565783</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>10080</v>
-      </c>
-      <c r="C5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.4986111111111111</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>3.838020651195538</v>
-      </c>
-      <c r="J5" t="n">
-        <v>1.948375887232062</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>10416</v>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.7943548387096774</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.04435483870967742</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.9556451612903226</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>3.493724205596369</v>
-      </c>
-      <c r="J6" t="n">
-        <v>1.52112615366548</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>10416</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.967741935483871</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.02956989247311828</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.9489247311827957</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.0510752688172043</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>3.139054811760477</v>
-      </c>
-      <c r="J7" t="n">
-        <v>1.762874770069682</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>9408</v>
-      </c>
-      <c r="C8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>2.346677582126682</v>
-      </c>
-      <c r="J8" t="n">
-        <v>1.227866562768589</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>10416</v>
-      </c>
-      <c r="C9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>2.146922001795506</v>
-      </c>
-      <c r="J9" t="n">
-        <v>1.113310072471372</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>4368</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0.9935897435897436</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="n">
-        <v>2.150312735372347</v>
-      </c>
-      <c r="J10" t="n">
-        <v>1.072085936102996</v>
+        <v>0.01666666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -3092,12 +2791,384 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>sensor_hours</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>raw_score_coverage</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>report_score_coverage</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ood_rate</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>L1_rate</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>L2_rate</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>L3_rate</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>D5_raw_median</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>D5_raw_p05</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>10416</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.9731182795698925</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.9005376344086021</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.07258064516129033</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.2142857142857143</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3.803353078474338</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1.97904518140716</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>10080</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.9722222222222222</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.8347222222222223</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.1375</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.8172619047619047</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.1827380952380952</v>
+      </c>
+      <c r="I3" t="n">
+        <v>3.372117688407658</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1.617424389235149</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>10416</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.2083333333333333</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.9326036866359447</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.0673963133640553</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3.068031596388653</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1.458730046565783</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>10080</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.4986111111111111</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.5013888888888889</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3.838020651195538</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1.948375887232062</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>10416</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.7943548387096774</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.1827956989247312</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.04435483870967742</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.9556451612903226</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3.493724205596369</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1.52112615366548</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>10416</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.967741935483871</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.02956989247311828</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.0228494623655914</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.9489247311827957</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.0510752688172043</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>3.139054811760477</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1.762874770069682</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>9408</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.005952380952380952</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2.346677582126682</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1.227866562768589</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>10416</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.1290322580645161</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2.146922001795506</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1.113310072471372</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4368</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.9935897435897436</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.09935897435897435</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2.150312735372347</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1.072085936102996</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
           <t>retained_fraction</t>
         </is>
       </c>
@@ -3113,20 +3184,45 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>top1_ci95_low</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>top1_ci95_high</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>top2</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>mrr</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>n_trials</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>n_month_blocks</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>analysis_unit</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>ci_method</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>interpretation</t>
         </is>
@@ -3143,15 +3239,34 @@
         <v>0.6222222222222222</v>
       </c>
       <c r="D2" t="n">
+        <v>0.4833333333333333</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.7833333333333333</v>
+      </c>
+      <c r="F2" t="n">
         <v>0.8388888888888889</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>0.7527856402856403</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>180</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>injected_24h_window</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>blocked_month_cluster_bootstrap</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t>controlled_injection_risk_coverage_not_field_error_rate</t>
         </is>
@@ -3168,15 +3283,34 @@
         <v>0.5763888888888888</v>
       </c>
       <c r="D3" t="n">
+        <v>0.4833333333333333</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.7575757575757576</v>
+      </c>
+      <c r="F3" t="n">
         <v>0.8263888888888888</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>0.7235166453916454</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>144</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>injected_24h_window</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>blocked_month_cluster_bootstrap</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>controlled_injection_risk_coverage_not_field_error_rate</t>
         </is>
@@ -3193,15 +3327,34 @@
         <v>0.5092592592592593</v>
       </c>
       <c r="D4" t="n">
+        <v>0.3939393939393939</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.7333333333333333</v>
+      </c>
+      <c r="F4" t="n">
         <v>0.7870370370370371</v>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
         <v>0.6761486969820303</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
         <v>108</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>injected_24h_window</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>blocked_month_cluster_bootstrap</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>controlled_injection_risk_coverage_not_field_error_rate</t>
         </is>
@@ -3218,15 +3371,34 @@
         <v>0.4722222222222222</v>
       </c>
       <c r="D5" t="n">
+        <v>0.2916666666666667</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.7222222222222222</v>
+      </c>
+      <c r="F5" t="n">
         <v>0.75</v>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
         <v>0.6477157102157103</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>72</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="I5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>injected_24h_window</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>blocked_month_cluster_bootstrap</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>controlled_injection_risk_coverage_not_field_error_rate</t>
         </is>

</xml_diff>